<commit_message>
New profile photo; blog: verified conversions, non-brand clicks over time, no impressions-bug mentions, round author photo; template updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Rt4pTaeDgP4WM14BDna8Z
</commit_message>
<xml_diff>
--- a/public/downloads/seo-report-template-q7m2x9.xlsx
+++ b/public/downloads/seo-report-template-q7m2x9.xlsx
@@ -527,7 +527,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>To my SEO: please fill in the yellow cells with every monthly report, and compare with the same month last year.</t>
+          <t>To my SEO: please fill in the yellow cells with every monthly report, and compare with an earlier period (the same month last year if you have it).</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Same month last year</t>
+          <t>Earlier period</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -646,7 +646,7 @@
       <c r="F8" s="8" t="n"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Up vs last year</t>
+          <t>Rising over time</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       <c r="F11" s="8" t="n"/>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Up vs last year</t>
+          <t>Rising over time</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Leads and sales from organic search, and how you verified them</t>
+          <t>Verified conversions from organic search (leads, bookings, sales) and how you verified them</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -771,7 +771,7 @@
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Up vs last year</t>
+          <t>Rising over time</t>
         </is>
       </c>
     </row>
@@ -789,13 +789,6 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Use clicks, not impressions: Google misreported impressions from May 2025 to April 2026.</t>
-        </is>
-      </c>
-    </row>
     <row r="19">
       <c r="B19" s="9" t="inlineStr">
         <is>
@@ -818,9 +811,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="B16:G16"/>
-    <mergeCell ref="B17:G17"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId1"/>

</xml_diff>